<commit_message>
feat(affiliate): add iPhone 15-18 Apple Flagship Store products
</commit_message>
<xml_diff>
--- a/affiliate_products.xlsx
+++ b/affiliate_products.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="390" yWindow="615" windowWidth="13095" windowHeight="7620" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Affiliate Products" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Affiliate Products" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -507,7 +507,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -1713,6 +1713,146 @@
       <c r="F33" t="inlineStr">
         <is>
           <t>กระดาษทิชชู่ PASEO เบบี้เพียว หนา 3 ชั้น สัมผัสนุ่มละมุน อ่อนโยนต่อผิว ยกลังสุดคุ้ม</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>17</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Apple iPhone 18 Pro Max (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8AWCoHKL6C</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Apple iPhone 18 Pro Max ชิป A20 Pro กล้องซูมคมชัด ดีไซน์พรีเมียม สั่งซื้อผ่าน Apple Flagship Store ของแท้ 100% พร้อมรับสิทธิ์ผ่อน 0% SpayLater</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztn-msxxsasoiscl48</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>18</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Apple iPhone 17 Pro (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/5AsbEphgh5</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Apple iPhone 17 Pro ชิป A19 Pro หน้าจอ ProMotion 120Hz แบตเตอรี่อึดยิ่งขึ้น ระบบกล้องโปร เครื่องศูนย์แท้พร้อมประกันศูนย์ไทย 1 ปีเต็ม</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztf-msuyb0tv79qff4</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>19</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Apple iPhone 16 Plus (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/LnLTzHQeV</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Apple iPhone 16 Plus จอใหญ่เต็มตา แบตเตอรี่อึดทนทาน รองรับ Apple Intelligence เต็มรูปแบบ ชิป A18 เครื่องศูนย์ไทยแท้ ผ่อน 0% ได้</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>https://down-th.img.susercontent.com/file/th-11134207-81ztg-msuy0uk4gkjo7b</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>20</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Apple iPhone 15 (เครื่องศูนย์ไทย ประกันศูนย์ 1 ปี) Shopee Mall</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>https://s.shopee.co.th/8fSTPKxXrZ</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>xxx</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Apple iPhone 15 พอร์ต USB-C กล้องหลัก 48MP หน้าจอ Dynamic Island สุดคุ้มค่า ใช้งานลื่นไหลยาวนาน เครื่องศูนย์ไทยแท้</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>https://store.storeimages.cdn-apple.com/8756/as-images.apple.com/is/iphone-15-finish-select-202309-6-1inch-black?wid=5120&amp;hei=2880&amp;fmt=p-jpg&amp;qlt=80&amp;.v=1692923777972</t>
         </is>
       </c>
     </row>

</xml_diff>